<commit_message>
Farhanfeat(categoriser): rename "Gifts & Outing" -> "Outings", add Personal Care
- rename the "Gifts  & Outing" category to "Outings" everywhere it is
  referenced: categories.json, nswtg_rollup.json (annual + plan rollups),
  forecast_benchmarks.json seasonality flags, and the monthly template
- add a new "Personal Care" expense category (unmapped personal-living line)
- expand merchant patterns from triage (Groceries, Fast food, Medicine,
  Rent -> GOODWILL CARE, etc.) and normalise the JSON to one pattern per line
- forecast benchmarks: Rent now $1,000/month to GOODWILL CARE ($12,000/yr);
  DSP reason notes the one-off backpay lump sum excluded from the forecast
- update categoriser + annual-accounts artifact tests for the new names
</commit_message>
<xml_diff>
--- a/templates/monthly_template.xlsx
+++ b/templates/monthly_template.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="StartingBalance">Summary!$L$8</definedName>
@@ -627,9 +627,7 @@
     <xf numFmtId="164" fontId="17" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="bottom"/>
@@ -1508,7 +1506,7 @@
       <c r="I12" s="34" t="n"/>
       <c r="J12" s="34" t="n"/>
       <c r="K12" s="34" t="n"/>
-      <c r="L12" s="35" t="n"/>
+      <c r="L12" s="44" t="n"/>
       <c r="M12" s="22" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1" s="149">
@@ -1523,7 +1521,7 @@
         <f>iferror(E17/D17-1, "")</f>
         <v/>
       </c>
-      <c r="L13" s="35" t="n"/>
+      <c r="L13" s="44" t="n"/>
       <c r="M13" s="39" t="n"/>
     </row>
     <row r="14" ht="24" customHeight="1" s="149">
@@ -1540,7 +1538,7 @@
       </c>
       <c r="J14" s="151" t="n"/>
       <c r="K14" s="151" t="n"/>
-      <c r="L14" s="35" t="n"/>
+      <c r="L14" s="44" t="n"/>
       <c r="M14" s="42" t="n"/>
     </row>
     <row r="15" ht="39.75" customHeight="1" s="149">
@@ -1579,7 +1577,7 @@
         <f>if(J15&lt;0, "Spent this month", "Saved this month")</f>
         <v/>
       </c>
-      <c r="L16" s="35" t="n"/>
+      <c r="L16" s="44" t="n"/>
       <c r="M16" s="50" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1" s="149">
@@ -1598,7 +1596,7 @@
       <c r="G17" s="36" t="n"/>
       <c r="H17" s="33" t="n"/>
       <c r="I17" s="34" t="n"/>
-      <c r="L17" s="35" t="n"/>
+      <c r="L17" s="44" t="n"/>
       <c r="M17" s="22" t="n"/>
     </row>
     <row r="18" ht="12" customHeight="1" s="149">
@@ -2123,7 +2121,7 @@
       <c r="A35" s="108" t="n"/>
       <c r="B35" s="156" t="inlineStr">
         <is>
-          <t>Gifts  &amp; Outing</t>
+          <t>Outings</t>
         </is>
       </c>
       <c r="C35" s="157" t="n"/>

</xml_diff>